<commit_message>
ML models and master runner added to CI/CD pipeline
</commit_message>
<xml_diff>
--- a/reports/anomaly_detection_report.xlsx
+++ b/reports/anomaly_detection_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Critical Anomalies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Warning Anomalies" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Department Benchmarks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Underperforming Branch Dept" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critical Anomalies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warning Anomalies" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Department Benchmarks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Underperforming Branch Dept" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,42 +432,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>branch</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dept_avg_margin</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>z_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>revenue_impact</t>
         </is>
@@ -1326,42 +1338,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>product_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>branch</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dept_avg_margin</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>z_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>revenue_impact</t>
         </is>
@@ -5564,27 +5576,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>dept_avg_margin</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>dept_std_margin</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>dept_median_margin</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dept_product_count</t>
         </is>
@@ -6080,27 +6092,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>branch</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>avg_margin</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>dept_avg</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>gap</t>
         </is>

</xml_diff>